<commit_message>
updated to fix bugs
updated to fix bugs
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_PWR_RES_MustRun.xlsx
+++ b/SuppXLS/Scen_PWR_RES_MustRun.xlsx
@@ -13204,11 +13204,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ANNUAL</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>UP</t>
@@ -13216,7 +13211,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NCAP_AF</t>
+          <t>NCAP_AFA</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -13235,11 +13230,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ANNUAL</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>UP</t>
@@ -13247,7 +13237,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NCAP_AF</t>
+          <t>NCAP_AFA</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -13266,11 +13256,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ANNUAL</t>
-        </is>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>UP</t>
@@ -13278,7 +13263,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NCAP_AF</t>
+          <t>NCAP_AFA</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -13297,11 +13282,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ANNUAL</t>
-        </is>
-      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>UP</t>
@@ -13309,7 +13289,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NCAP_AF</t>
+          <t>NCAP_AFA</t>
         </is>
       </c>
       <c r="E6" t="n">

</xml_diff>